<commit_message>
Sign-in screens: share the snapshot split-panel hero
Move the snapshot hero panel and signal field to components/brand-hero
as a prop-driven HeroPanel, and use it in the (auth) layout so /login,
check-email and magic-link verify match the snapshot intake screen.
Restyle the three auth steps to fit the new frame; drop the disabled
Google sign-in placeholder; point legal links at the marketing site.

Co-Authored-By: Claude Opus 5.5 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/feature-test-tracker.xlsx
+++ b/feature-test-tracker.xlsx
@@ -15,7 +15,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="416" uniqueCount="148">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="460" uniqueCount="161">
   <si>
     <t>Phase</t>
   </si>
@@ -405,6 +405,45 @@
   </si>
   <si>
     <t>Page frame verified; report data not fetched locally (API not running → expected error panel).</t>
+  </si>
+  <si>
+    <t>/login redesign — shared hero, 0 console errors (1440, 1280 dark, 390 mobile; 0px overflow)</t>
+  </si>
+  <si>
+    <t>Headless Chrome against next dev.</t>
+  </si>
+  <si>
+    <t>/login — invalid email shows inline error with red border</t>
+  </si>
+  <si>
+    <t/>
+  </si>
+  <si>
+    <t>/login → POST /auth/magic-link → /login/check-email</t>
+  </si>
+  <si>
+    <t>200 (mocked)</t>
+  </si>
+  <si>
+    <t>API response mocked (local API not running); navigation + check-email render verified.</t>
+  </si>
+  <si>
+    <t>/auth/magic-link/verify without token → error state with 'Request a new link'</t>
+  </si>
+  <si>
+    <t>Duplicate back-to-login link removed.</t>
+  </si>
+  <si>
+    <t>Login Terms / Privacy links</t>
+  </si>
+  <si>
+    <t>Were /terms and /privacy-policy on the app domain (404). Now bebestwithai.com/terms.html and /privacy-policy.html (both 200).</t>
+  </si>
+  <si>
+    <t>Disabled 'Continue with Google' button removed</t>
+  </si>
+  <si>
+    <t>Was a permanently disabled, unwired control (TODO in code).</t>
   </si>
   <si>
     <t>BeBest Platform — Customer Journey Test Results (2026-09-06)</t>
@@ -869,7 +908,7 @@
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
   </sheetPr>
-  <dimension ref="A1:H55"/>
+  <dimension ref="A1:H61"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="0"/>
   <cols>
     <col min="1" max="1" width="8" customWidth="1"/>
@@ -2215,6 +2254,150 @@
         <v>14</v>
       </c>
       <c r="H55" s="2" t="s">
+        <v>117</v>
+      </c>
+    </row>
+    <row r="56" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A56" s="2" t="s">
+        <v>42</v>
+      </c>
+      <c r="B56" s="2" t="s">
+        <v>43</v>
+      </c>
+      <c r="C56" s="2" t="s">
+        <v>130</v>
+      </c>
+      <c r="D56" s="3" t="s">
+        <v>11</v>
+      </c>
+      <c r="E56" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="F56" s="2" t="s">
+        <v>131</v>
+      </c>
+      <c r="G56" s="2" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="57" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A57" s="2" t="s">
+        <v>42</v>
+      </c>
+      <c r="B57" s="2" t="s">
+        <v>43</v>
+      </c>
+      <c r="C57" s="2" t="s">
+        <v>132</v>
+      </c>
+      <c r="D57" s="3" t="s">
+        <v>11</v>
+      </c>
+      <c r="E57" s="2" t="s">
+        <v>121</v>
+      </c>
+      <c r="F57" s="2" t="s">
+        <v>133</v>
+      </c>
+      <c r="G57" s="2" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="58" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A58" s="2" t="s">
+        <v>42</v>
+      </c>
+      <c r="B58" s="2" t="s">
+        <v>43</v>
+      </c>
+      <c r="C58" s="2" t="s">
+        <v>134</v>
+      </c>
+      <c r="D58" s="3" t="s">
+        <v>11</v>
+      </c>
+      <c r="E58" s="2" t="s">
+        <v>135</v>
+      </c>
+      <c r="F58" s="2" t="s">
+        <v>136</v>
+      </c>
+      <c r="G58" s="2" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="59" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A59" s="2" t="s">
+        <v>42</v>
+      </c>
+      <c r="B59" s="2" t="s">
+        <v>43</v>
+      </c>
+      <c r="C59" s="2" t="s">
+        <v>137</v>
+      </c>
+      <c r="D59" s="3" t="s">
+        <v>11</v>
+      </c>
+      <c r="E59" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="F59" s="2" t="s">
+        <v>138</v>
+      </c>
+      <c r="G59" s="2" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="60" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A60" s="2" t="s">
+        <v>42</v>
+      </c>
+      <c r="B60" s="2" t="s">
+        <v>43</v>
+      </c>
+      <c r="C60" s="2" t="s">
+        <v>139</v>
+      </c>
+      <c r="D60" s="3" t="s">
+        <v>11</v>
+      </c>
+      <c r="E60" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="F60" s="2" t="s">
+        <v>140</v>
+      </c>
+      <c r="G60" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="H60" s="2" t="s">
+        <v>117</v>
+      </c>
+    </row>
+    <row r="61" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A61" s="2" t="s">
+        <v>42</v>
+      </c>
+      <c r="B61" s="2" t="s">
+        <v>43</v>
+      </c>
+      <c r="C61" s="2" t="s">
+        <v>141</v>
+      </c>
+      <c r="D61" s="3" t="s">
+        <v>11</v>
+      </c>
+      <c r="E61" s="2" t="s">
+        <v>121</v>
+      </c>
+      <c r="F61" s="2" t="s">
+        <v>142</v>
+      </c>
+      <c r="G61" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="H61" s="2" t="s">
         <v>117</v>
       </c>
     </row>
@@ -2237,15 +2420,15 @@
   <sheetData>
     <row r="1" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A1" s="5" t="s">
-        <v>130</v>
+        <v>143</v>
       </c>
     </row>
     <row r="3" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>131</v>
+        <v>144</v>
       </c>
       <c r="B3">
-        <v>54</v>
+        <v>60</v>
       </c>
     </row>
     <row r="4" spans="1:2" x14ac:dyDescent="0.25">
@@ -2253,12 +2436,12 @@
         <v>11</v>
       </c>
       <c r="B4">
-        <v>54</v>
+        <v>60</v>
       </c>
     </row>
     <row r="5" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>132</v>
+        <v>145</v>
       </c>
       <c r="B5">
         <v>0</v>
@@ -2266,7 +2449,7 @@
     </row>
     <row r="6" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>133</v>
+        <v>146</v>
       </c>
       <c r="B6">
         <v>0</v>
@@ -2274,7 +2457,7 @@
     </row>
     <row r="7" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>134</v>
+        <v>147</v>
       </c>
       <c r="B7">
         <v>4</v>
@@ -2282,68 +2465,68 @@
     </row>
     <row r="9" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
-        <v>135</v>
+        <v>148</v>
       </c>
     </row>
     <row r="10" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
-        <v>136</v>
+        <v>149</v>
       </c>
       <c r="B10" t="s">
-        <v>137</v>
+        <v>150</v>
       </c>
     </row>
     <row r="11" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
-        <v>138</v>
+        <v>151</v>
       </c>
       <c r="B11" t="s">
-        <v>137</v>
+        <v>150</v>
       </c>
     </row>
     <row r="12" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
-        <v>139</v>
+        <v>152</v>
       </c>
       <c r="B12" t="s">
-        <v>137</v>
+        <v>150</v>
       </c>
     </row>
     <row r="13" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
-        <v>140</v>
+        <v>153</v>
       </c>
       <c r="B13" t="s">
-        <v>137</v>
+        <v>150</v>
       </c>
     </row>
     <row r="15" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
-        <v>141</v>
+        <v>154</v>
       </c>
     </row>
     <row r="16" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
-        <v>142</v>
+        <v>155</v>
       </c>
       <c r="B16" t="s">
-        <v>143</v>
+        <v>156</v>
       </c>
     </row>
     <row r="17" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
-        <v>144</v>
+        <v>157</v>
       </c>
       <c r="B17" t="s">
-        <v>145</v>
+        <v>158</v>
       </c>
     </row>
     <row r="18" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
-        <v>146</v>
+        <v>159</v>
       </c>
       <c r="B18" t="s">
-        <v>147</v>
+        <v>160</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Epic 22 Phase 1 frontend: Platform view screens; session.md and tracker
/platform overview (KPIs + live capability matrix), organizations and
cross-tenant org detail, users (admin sign-in link), agencies, growth
(existing CRM screens reused under /platform/growth via a base-path
provider, plus snapshot requests), operations (stuck filter, admin
cancel with 409 handling) and audit log. Loading/empty/503/403 states,
light and dark, 390px.

Verified on a production build against the dev API and database:
browser walk 63/63, smoke:platform 98/98; typecheck and build clean.

Co-Authored-By: Claude Opus 5.5 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/feature-test-tracker.xlsx
+++ b/feature-test-tracker.xlsx
@@ -15,7 +15,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="517" uniqueCount="177">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="581" uniqueCount="195">
   <si>
     <t>Phase</t>
   </si>
@@ -492,6 +492,60 @@
   </si>
   <si>
     <t>Role re-read from DB per request.</t>
+  </si>
+  <si>
+    <t>Platform View</t>
+  </si>
+  <si>
+    <t>/platform overview KPIs + live capability matrix (25 capabilities, live dependency checks)</t>
+  </si>
+  <si>
+    <t>Browser walk 63/63 on a production build vs dev API+DB.</t>
+  </si>
+  <si>
+    <t>Organizations list (search/filters) + cross-tenant org detail (usage vs limits, members, runs, audit)</t>
+  </si>
+  <si>
+    <t>Staff not a member of the org.</t>
+  </si>
+  <si>
+    <t>Users list + detail; admin 'Send sign-in link' (support disabled)</t>
+  </si>
+  <si>
+    <t>Agencies + clients</t>
+  </si>
+  <si>
+    <t>Growth: CRM leads/deals/accounts inside Platform view for staff + snapshot requests</t>
+  </si>
+  <si>
+    <t>CRM now admits platform staff (support=analyst, admin=admin).</t>
+  </si>
+  <si>
+    <t>Operations: cross-org jobs, stuck filter, admin cancel (409 when already finished)</t>
+  </si>
+  <si>
+    <t>200/409</t>
+  </si>
+  <si>
+    <t>DB row verified cancelled; audit row written.</t>
+  </si>
+  <si>
+    <t>Audit log: app + platform events, filters, expandable details</t>
+  </si>
+  <si>
+    <t>Customer: all /platform/* routes redirect, every /api/platform/* call 403 with no access row</t>
+  </si>
+  <si>
+    <t>403</t>
+  </si>
+  <si>
+    <t>smoke:platform 98/98.</t>
+  </si>
+  <si>
+    <t>writeAuditEvent: org-less audit rows (login/logout/apply) were silently dropped under bebest_app</t>
+  </si>
+  <si>
+    <t>create() RETURNING blocked by read policy; now createMany.</t>
   </si>
   <si>
     <t>BeBest Platform — Customer Journey Test Results (2026-09-06)</t>
@@ -956,7 +1010,7 @@
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
   </sheetPr>
-  <dimension ref="A1:H69"/>
+  <dimension ref="A1:H78"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="0"/>
   <cols>
     <col min="1" max="1" width="8" customWidth="1"/>
@@ -2634,6 +2688,216 @@
       </c>
       <c r="G69" s="2" t="s">
         <v>14</v>
+      </c>
+    </row>
+    <row r="70" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A70" s="2" t="s">
+        <v>64</v>
+      </c>
+      <c r="B70" s="2" t="s">
+        <v>159</v>
+      </c>
+      <c r="C70" s="2" t="s">
+        <v>160</v>
+      </c>
+      <c r="D70" s="3" t="s">
+        <v>11</v>
+      </c>
+      <c r="E70" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="F70" s="2" t="s">
+        <v>161</v>
+      </c>
+      <c r="G70" s="2" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="71" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A71" s="2" t="s">
+        <v>64</v>
+      </c>
+      <c r="B71" s="2" t="s">
+        <v>159</v>
+      </c>
+      <c r="C71" s="2" t="s">
+        <v>162</v>
+      </c>
+      <c r="D71" s="3" t="s">
+        <v>11</v>
+      </c>
+      <c r="E71" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="F71" s="2" t="s">
+        <v>163</v>
+      </c>
+      <c r="G71" s="2" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="72" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A72" s="2" t="s">
+        <v>64</v>
+      </c>
+      <c r="B72" s="2" t="s">
+        <v>159</v>
+      </c>
+      <c r="C72" s="2" t="s">
+        <v>164</v>
+      </c>
+      <c r="D72" s="3" t="s">
+        <v>11</v>
+      </c>
+      <c r="E72" s="2" t="s">
+        <v>157</v>
+      </c>
+      <c r="F72" s="2" t="s">
+        <v>133</v>
+      </c>
+      <c r="G72" s="2" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="73" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A73" s="2" t="s">
+        <v>64</v>
+      </c>
+      <c r="B73" s="2" t="s">
+        <v>159</v>
+      </c>
+      <c r="C73" s="2" t="s">
+        <v>165</v>
+      </c>
+      <c r="D73" s="3" t="s">
+        <v>11</v>
+      </c>
+      <c r="E73" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="F73" s="2" t="s">
+        <v>133</v>
+      </c>
+      <c r="G73" s="2" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="74" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A74" s="2" t="s">
+        <v>64</v>
+      </c>
+      <c r="B74" s="2" t="s">
+        <v>159</v>
+      </c>
+      <c r="C74" s="2" t="s">
+        <v>166</v>
+      </c>
+      <c r="D74" s="3" t="s">
+        <v>11</v>
+      </c>
+      <c r="E74" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="F74" s="2" t="s">
+        <v>167</v>
+      </c>
+      <c r="G74" s="2" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="75" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A75" s="2" t="s">
+        <v>64</v>
+      </c>
+      <c r="B75" s="2" t="s">
+        <v>159</v>
+      </c>
+      <c r="C75" s="2" t="s">
+        <v>168</v>
+      </c>
+      <c r="D75" s="3" t="s">
+        <v>11</v>
+      </c>
+      <c r="E75" s="2" t="s">
+        <v>169</v>
+      </c>
+      <c r="F75" s="2" t="s">
+        <v>170</v>
+      </c>
+      <c r="G75" s="2" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="76" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A76" s="2" t="s">
+        <v>64</v>
+      </c>
+      <c r="B76" s="2" t="s">
+        <v>159</v>
+      </c>
+      <c r="C76" s="2" t="s">
+        <v>171</v>
+      </c>
+      <c r="D76" s="3" t="s">
+        <v>11</v>
+      </c>
+      <c r="E76" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="F76" s="2" t="s">
+        <v>133</v>
+      </c>
+      <c r="G76" s="2" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="77" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A77" s="2" t="s">
+        <v>64</v>
+      </c>
+      <c r="B77" s="2" t="s">
+        <v>159</v>
+      </c>
+      <c r="C77" s="2" t="s">
+        <v>172</v>
+      </c>
+      <c r="D77" s="3" t="s">
+        <v>11</v>
+      </c>
+      <c r="E77" s="2" t="s">
+        <v>173</v>
+      </c>
+      <c r="F77" s="2" t="s">
+        <v>174</v>
+      </c>
+      <c r="G77" s="2" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="78" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A78" s="2" t="s">
+        <v>94</v>
+      </c>
+      <c r="B78" s="2" t="s">
+        <v>95</v>
+      </c>
+      <c r="C78" s="2" t="s">
+        <v>175</v>
+      </c>
+      <c r="D78" s="3" t="s">
+        <v>11</v>
+      </c>
+      <c r="E78" s="2" t="s">
+        <v>121</v>
+      </c>
+      <c r="F78" s="2" t="s">
+        <v>176</v>
+      </c>
+      <c r="G78" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="H78" s="2" t="s">
+        <v>117</v>
       </c>
     </row>
   </sheetData>
@@ -2655,15 +2919,15 @@
   <sheetData>
     <row r="1" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A1" s="5" t="s">
-        <v>159</v>
+        <v>177</v>
       </c>
     </row>
     <row r="3" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>160</v>
+        <v>178</v>
       </c>
       <c r="B3">
-        <v>68</v>
+        <v>77</v>
       </c>
     </row>
     <row r="4" spans="1:2" x14ac:dyDescent="0.25">
@@ -2671,12 +2935,12 @@
         <v>11</v>
       </c>
       <c r="B4">
-        <v>68</v>
+        <v>77</v>
       </c>
     </row>
     <row r="5" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>161</v>
+        <v>179</v>
       </c>
       <c r="B5">
         <v>0</v>
@@ -2684,7 +2948,7 @@
     </row>
     <row r="6" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>162</v>
+        <v>180</v>
       </c>
       <c r="B6">
         <v>0</v>
@@ -2692,7 +2956,7 @@
     </row>
     <row r="7" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>163</v>
+        <v>181</v>
       </c>
       <c r="B7">
         <v>4</v>
@@ -2700,68 +2964,68 @@
     </row>
     <row r="9" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
-        <v>164</v>
+        <v>182</v>
       </c>
     </row>
     <row r="10" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
-        <v>165</v>
+        <v>183</v>
       </c>
       <c r="B10" t="s">
-        <v>166</v>
+        <v>184</v>
       </c>
     </row>
     <row r="11" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
-        <v>167</v>
+        <v>185</v>
       </c>
       <c r="B11" t="s">
-        <v>166</v>
+        <v>184</v>
       </c>
     </row>
     <row r="12" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
-        <v>168</v>
+        <v>186</v>
       </c>
       <c r="B12" t="s">
-        <v>166</v>
+        <v>184</v>
       </c>
     </row>
     <row r="13" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
-        <v>169</v>
+        <v>187</v>
       </c>
       <c r="B13" t="s">
-        <v>166</v>
+        <v>184</v>
       </c>
     </row>
     <row r="15" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
-        <v>170</v>
+        <v>188</v>
       </c>
     </row>
     <row r="16" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
-        <v>171</v>
+        <v>189</v>
       </c>
       <c r="B16" t="s">
-        <v>172</v>
+        <v>190</v>
       </c>
     </row>
     <row r="17" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
-        <v>173</v>
+        <v>191</v>
       </c>
       <c r="B17" t="s">
-        <v>174</v>
+        <v>192</v>
       </c>
     </row>
     <row r="18" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
-        <v>175</v>
+        <v>193</v>
       </c>
       <c r="B18" t="s">
-        <v>176</v>
+        <v>194</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Epic 22 Phase 2 frontend: Organization view
Settings: Organization tab (rename, owner-only delete with typed
confirmation), real Notifications and Autonomy tabs, ?tab= deep links.
/invitations/accept (public; preview, sign-in round trip, accept, email
mismatch). First login relies on server slugs and routes by
needsOnboarding; onboarding completion is server-side and the Done step
shows the first crawl and query set. Agent card respects the org
autonomy limit.

Fixes: bell crash on invitation_accepted, Team tab loading the first org
instead of the active one, Overview flashing 'Start onboarding' while
the session loads (use-brand-profile derives loading), switcher lagging
a full /auth/me after rename (applyOrgRename).

Browser walk on a production build vs the dev API and DB: 48/50 (the
autonomy 422 path is unreachable on Free and was verified on Pro; the
rename timing check fixed and re-probed). smoke:org 98/98.

Co-Authored-By: Claude Opus 5.5 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/feature-test-tracker.xlsx
+++ b/feature-test-tracker.xlsx
@@ -15,7 +15,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="581" uniqueCount="195">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="663" uniqueCount="214">
   <si>
     <t>Phase</t>
   </si>
@@ -546,6 +546,63 @@
   </si>
   <si>
     <t>create() RETURNING blocked by read policy; now createMany.</t>
+  </si>
+  <si>
+    <t>First login: two users with the same email prefix get separate orgs (john-15/john-16), both routed to onboarding</t>
+  </si>
+  <si>
+    <t>Server-side unique slugs (race-safe).</t>
+  </si>
+  <si>
+    <t>Completion stored server-side; Done starts first crawl + creates active query set; idempotent; works after clearing localStorage / on a 2nd device</t>
+  </si>
+  <si>
+    <t>Browser walk vs dev DB; DB rows verified.</t>
+  </si>
+  <si>
+    <t>Done with steps missing lists them (422 onboarding_incomplete)</t>
+  </si>
+  <si>
+    <t>422</t>
+  </si>
+  <si>
+    <t>Invitation accept page: signed-out preview, sign-in returns to invite, accept joins org, inviter notified</t>
+  </si>
+  <si>
+    <t>Invite link previously 404'd.</t>
+  </si>
+  <si>
+    <t>Invitation opened by wrong account -&gt; email_mismatch, no membership</t>
+  </si>
+  <si>
+    <t>Settings &gt; Organization: rename (switcher updates immediately), audit row</t>
+  </si>
+  <si>
+    <t>Settings &gt; Organization: owner-only delete with typed confirmation; moved to remaining org</t>
+  </si>
+  <si>
+    <t>200/422</t>
+  </si>
+  <si>
+    <t>Soft delete.</t>
+  </si>
+  <si>
+    <t>Settings &gt; Notifications: per-event in-app/email toggles persist and are honoured by notify()</t>
+  </si>
+  <si>
+    <t>Settings &gt; Autonomy: org limit 1-3 (default 3, plan-capped); agent card disables higher levels; API 422 above limit</t>
+  </si>
+  <si>
+    <t>Free plan has no agents (402) — 422 path verified on Pro.</t>
+  </si>
+  <si>
+    <t>Overview no longer flashes 'Start onboarding' for set-up users while session loads</t>
+  </si>
+  <si>
+    <t>use-brand-profile derived loading.</t>
+  </si>
+  <si>
+    <t>Notification bell: invitation_accepted rendered (was React #130 crash)</t>
   </si>
   <si>
     <t>BeBest Platform — Customer Journey Test Results (2026-09-06)</t>
@@ -1010,7 +1067,7 @@
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
   </sheetPr>
-  <dimension ref="A1:H78"/>
+  <dimension ref="A1:H89"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="0"/>
   <cols>
     <col min="1" max="1" width="8" customWidth="1"/>
@@ -2897,6 +2954,274 @@
         <v>14</v>
       </c>
       <c r="H78" s="2" t="s">
+        <v>117</v>
+      </c>
+    </row>
+    <row r="79" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A79" s="2" t="s">
+        <v>42</v>
+      </c>
+      <c r="B79" s="2" t="s">
+        <v>43</v>
+      </c>
+      <c r="C79" s="2" t="s">
+        <v>177</v>
+      </c>
+      <c r="D79" s="3" t="s">
+        <v>11</v>
+      </c>
+      <c r="E79" s="2" t="s">
+        <v>110</v>
+      </c>
+      <c r="F79" s="2" t="s">
+        <v>178</v>
+      </c>
+      <c r="G79" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="H79" s="2" t="s">
+        <v>117</v>
+      </c>
+    </row>
+    <row r="80" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A80" s="2" t="s">
+        <v>55</v>
+      </c>
+      <c r="B80" s="2" t="s">
+        <v>56</v>
+      </c>
+      <c r="C80" s="2" t="s">
+        <v>179</v>
+      </c>
+      <c r="D80" s="3" t="s">
+        <v>11</v>
+      </c>
+      <c r="E80" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="F80" s="2" t="s">
+        <v>180</v>
+      </c>
+      <c r="G80" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="H80" s="2" t="s">
+        <v>117</v>
+      </c>
+    </row>
+    <row r="81" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A81" s="2" t="s">
+        <v>55</v>
+      </c>
+      <c r="B81" s="2" t="s">
+        <v>56</v>
+      </c>
+      <c r="C81" s="2" t="s">
+        <v>181</v>
+      </c>
+      <c r="D81" s="3" t="s">
+        <v>11</v>
+      </c>
+      <c r="E81" s="2" t="s">
+        <v>182</v>
+      </c>
+      <c r="F81" s="2" t="s">
+        <v>133</v>
+      </c>
+      <c r="G81" s="2" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="82" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A82" s="2" t="s">
+        <v>42</v>
+      </c>
+      <c r="B82" s="2" t="s">
+        <v>43</v>
+      </c>
+      <c r="C82" s="2" t="s">
+        <v>183</v>
+      </c>
+      <c r="D82" s="3" t="s">
+        <v>11</v>
+      </c>
+      <c r="E82" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="F82" s="2" t="s">
+        <v>184</v>
+      </c>
+      <c r="G82" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="H82" s="2" t="s">
+        <v>117</v>
+      </c>
+    </row>
+    <row r="83" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A83" s="2" t="s">
+        <v>42</v>
+      </c>
+      <c r="B83" s="2" t="s">
+        <v>43</v>
+      </c>
+      <c r="C83" s="2" t="s">
+        <v>185</v>
+      </c>
+      <c r="D83" s="3" t="s">
+        <v>11</v>
+      </c>
+      <c r="E83" s="2" t="s">
+        <v>173</v>
+      </c>
+      <c r="F83" s="2" t="s">
+        <v>133</v>
+      </c>
+      <c r="G83" s="2" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="84" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A84" s="2" t="s">
+        <v>64</v>
+      </c>
+      <c r="B84" s="2" t="s">
+        <v>65</v>
+      </c>
+      <c r="C84" s="2" t="s">
+        <v>186</v>
+      </c>
+      <c r="D84" s="3" t="s">
+        <v>11</v>
+      </c>
+      <c r="E84" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="F84" s="2" t="s">
+        <v>133</v>
+      </c>
+      <c r="G84" s="2" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="85" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A85" s="2" t="s">
+        <v>64</v>
+      </c>
+      <c r="B85" s="2" t="s">
+        <v>65</v>
+      </c>
+      <c r="C85" s="2" t="s">
+        <v>187</v>
+      </c>
+      <c r="D85" s="3" t="s">
+        <v>11</v>
+      </c>
+      <c r="E85" s="2" t="s">
+        <v>188</v>
+      </c>
+      <c r="F85" s="2" t="s">
+        <v>189</v>
+      </c>
+      <c r="G85" s="2" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="86" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A86" s="2" t="s">
+        <v>64</v>
+      </c>
+      <c r="B86" s="2" t="s">
+        <v>65</v>
+      </c>
+      <c r="C86" s="2" t="s">
+        <v>190</v>
+      </c>
+      <c r="D86" s="3" t="s">
+        <v>11</v>
+      </c>
+      <c r="E86" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="F86" s="2" t="s">
+        <v>133</v>
+      </c>
+      <c r="G86" s="2" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="87" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A87" s="2" t="s">
+        <v>64</v>
+      </c>
+      <c r="B87" s="2" t="s">
+        <v>65</v>
+      </c>
+      <c r="C87" s="2" t="s">
+        <v>191</v>
+      </c>
+      <c r="D87" s="3" t="s">
+        <v>11</v>
+      </c>
+      <c r="E87" s="2" t="s">
+        <v>188</v>
+      </c>
+      <c r="F87" s="2" t="s">
+        <v>192</v>
+      </c>
+      <c r="G87" s="2" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="88" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A88" s="2" t="s">
+        <v>64</v>
+      </c>
+      <c r="B88" s="2" t="s">
+        <v>65</v>
+      </c>
+      <c r="C88" s="2" t="s">
+        <v>193</v>
+      </c>
+      <c r="D88" s="3" t="s">
+        <v>11</v>
+      </c>
+      <c r="E88" s="2" t="s">
+        <v>121</v>
+      </c>
+      <c r="F88" s="2" t="s">
+        <v>194</v>
+      </c>
+      <c r="G88" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="H88" s="2" t="s">
+        <v>117</v>
+      </c>
+    </row>
+    <row r="89" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A89" s="2" t="s">
+        <v>64</v>
+      </c>
+      <c r="B89" s="2" t="s">
+        <v>65</v>
+      </c>
+      <c r="C89" s="2" t="s">
+        <v>195</v>
+      </c>
+      <c r="D89" s="3" t="s">
+        <v>11</v>
+      </c>
+      <c r="E89" s="2" t="s">
+        <v>121</v>
+      </c>
+      <c r="F89" s="2" t="s">
+        <v>133</v>
+      </c>
+      <c r="G89" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="H89" s="2" t="s">
         <v>117</v>
       </c>
     </row>
@@ -2919,15 +3244,15 @@
   <sheetData>
     <row r="1" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A1" s="5" t="s">
-        <v>177</v>
+        <v>196</v>
       </c>
     </row>
     <row r="3" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>178</v>
+        <v>197</v>
       </c>
       <c r="B3">
-        <v>77</v>
+        <v>88</v>
       </c>
     </row>
     <row r="4" spans="1:2" x14ac:dyDescent="0.25">
@@ -2935,12 +3260,12 @@
         <v>11</v>
       </c>
       <c r="B4">
-        <v>77</v>
+        <v>88</v>
       </c>
     </row>
     <row r="5" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>179</v>
+        <v>198</v>
       </c>
       <c r="B5">
         <v>0</v>
@@ -2948,7 +3273,7 @@
     </row>
     <row r="6" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>180</v>
+        <v>199</v>
       </c>
       <c r="B6">
         <v>0</v>
@@ -2956,7 +3281,7 @@
     </row>
     <row r="7" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>181</v>
+        <v>200</v>
       </c>
       <c r="B7">
         <v>4</v>
@@ -2964,68 +3289,68 @@
     </row>
     <row r="9" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
-        <v>182</v>
+        <v>201</v>
       </c>
     </row>
     <row r="10" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
-        <v>183</v>
+        <v>202</v>
       </c>
       <c r="B10" t="s">
-        <v>184</v>
+        <v>203</v>
       </c>
     </row>
     <row r="11" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
-        <v>185</v>
+        <v>204</v>
       </c>
       <c r="B11" t="s">
-        <v>184</v>
+        <v>203</v>
       </c>
     </row>
     <row r="12" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
-        <v>186</v>
+        <v>205</v>
       </c>
       <c r="B12" t="s">
-        <v>184</v>
+        <v>203</v>
       </c>
     </row>
     <row r="13" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
-        <v>187</v>
+        <v>206</v>
       </c>
       <c r="B13" t="s">
-        <v>184</v>
+        <v>203</v>
       </c>
     </row>
     <row r="15" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
-        <v>188</v>
+        <v>207</v>
       </c>
     </row>
     <row r="16" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
-        <v>189</v>
+        <v>208</v>
       </c>
       <c r="B16" t="s">
-        <v>190</v>
+        <v>209</v>
       </c>
     </row>
     <row r="17" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
-        <v>191</v>
+        <v>210</v>
       </c>
       <c r="B17" t="s">
-        <v>192</v>
+        <v>211</v>
       </c>
     </row>
     <row r="18" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
-        <v>193</v>
+        <v>212</v>
       </c>
       <c r="B18" t="s">
-        <v>194</v>
+        <v>213</v>
       </c>
     </row>
   </sheetData>

</xml_diff>